<commit_message>
FR 3 and 4 added to Excel.
</commit_message>
<xml_diff>
--- a/Raport_gr3_pokoj4.xlsx
+++ b/Raport_gr3_pokoj4.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Raport z testów" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="94">
   <si>
     <t xml:space="preserve">Raport z testów</t>
   </si>
@@ -235,10 +235,10 @@
     <t xml:space="preserve">Testowany produkt, wersja</t>
   </si>
   <si>
+    <t xml:space="preserve">1.0.0</t>
+  </si>
+  <si>
     <t xml:space="preserve">Środowisko testowe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opis błędu</t>
   </si>
   <si>
     <r>
@@ -249,7 +249,9 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">System nie blokuje transferu TCP powyżej dozwolonej prędkości (100 Mbps). Zamiast zwrócić błąd walidacji (HTTP 422), operacja kończy się sukcesem (HTTP 200), </t>
+      <t xml:space="preserve">Serwer: uruchomiony w kontenerze Docker 
+Klient: testy automatyczne wykonywane w Robot Framework
+Werjsa OS: Arch Linus (rolling release) </t>
     </r>
     <r>
       <rPr>
@@ -258,8 +260,58 @@
         <rFont val="Arial"/>
         <family val="0"/>
       </rPr>
-      <t xml:space="preserve">I transfer przechodzi bez przeszkód</t>
+      <t xml:space="preserve"> Werjsa Kernel: Linux 6.19.6-arch1-1
+Wersja Dockera: Docker version 29.3.0, build 5927d80c76</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Opis błędu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">System nie blokuje transferu TCP powyżej dozwolonej prędkości (100 Mbps). Zamiast zwrócić błąd walidacji (HTTP 422), operacja kończy się sukcesem (HTTP 200), I transfer przechodzi bez przeszkód co oznacza niezgodność z załorzeniami projektu co do limitu prędkości.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kroki / scenariusz, podczas których  został wykryty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Ustawić prędkość transferu na 101+ Mbps 
+2. Ustawić protokół UDP 
+3. Wykonać transfer danych 
+4. Sprawdzić kod odpowiedzi HTTP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oczekiwany rezultat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTP Response Code  422</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uzyskany rezultat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTP Response Code 200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Powtarzalność</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Podjęte kroki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zweryfikowano konfigurację limitu prędkości 
+Powtórzono test wielokrotnie 
+Sprawdzono różne wartości powyżej limitu (np. 102, 110, 120, 220 Mbps – ten sam wynik)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analiza testera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prawdopodobny brak walidacji limitu prędkości po stronie backendu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Załączniki (logi/ zrzut z ekranu)</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="12"/>
@@ -268,59 +320,48 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve"> co oznacza niezgodność z załorzeniami projektu co do limitu prędkości.</t>
+      <t xml:space="preserve">Logi można znaleść w katalogu </t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Kroki / scenariusz, podczas których  został wykryty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oczekiwany rezultat</t>
-  </si>
-  <si>
     <r>
       <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
+        <i val="true"/>
+        <sz val="12"/>
+        <color rgb="FF333333"/>
         <rFont val="Arial"/>
         <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">HTTP Response Code </t>
+      <t xml:space="preserve">StartAndBeginTestOutput/</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">UDP transfer above allowed speed returns 200 instead of 422</t>
+  </si>
+  <si>
+    <t xml:space="preserve">System nie blokuje transferu UDP powyżej dozwolonej prędkości (100 Mbps). Zamiast zwrócić błąd walidacji (HTTP 422), operacja kończy się sukcesem (HTTP 200) I transfer przechodzi bez przeszkód, co oznacza niezgodność z załorzeniami projektu co do limitu prędkości.</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
-        <family val="0"/>
+        <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve"> 422</t>
+      <t xml:space="preserve">Logi można znaleść w katalogu </t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Uzyskany rezultat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HTTP Response Code 200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Powtarzalność</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Podjęte kroki</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analiza testera</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Załączniki (logi/ zrzut z ekranu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UDP transfer above allowed speed returns 200 instead of 422</t>
-  </si>
-  <si>
-    <t xml:space="preserve">System nie blokuje transferu UDP powyżej dozwolonej prędkości (100 Mbps). Zamiast zwrócić błąd walidacji (HTTP 422), operacja kończy się sukcesem (HTTP 200) I transfer przechodzi bez przeszkód, co oznacza niezgodność z załorzeniami projektu co do limitu prędkości.</t>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="12"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">StartAndBeginTestOutput/</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">no run</t>
@@ -341,7 +382,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -416,13 +457,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
-      <sz val="10"/>
-      <color rgb="FF1155CC"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="10.5"/>
       <color rgb="FF000000"/>
@@ -441,13 +475,37 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -475,7 +533,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -590,16 +648,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -607,95 +669,127 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -738,7 +832,7 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="00FFFFFF"/>
+        <color rgb="FFFFFFFF"/>
       </font>
       <fill>
         <patternFill>
@@ -750,7 +844,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFF2F2F2"/>
+      <rgbColor rgb="FFFFFFFF"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -767,7 +861,7 @@
       <rgbColor rgb="FF7F7F7F"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFF2F2F2"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -991,680 +1085,680 @@
   <dimension ref="A1:I28"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="56.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="29.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="56.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="29.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="2" t="s">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-    </row>
-    <row r="4" customFormat="false" ht="25.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="5" t="s">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="7" t="s">
+      <c r="D5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="7" t="s">
+      <c r="D6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="7" t="s">
+      <c r="D7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="9"/>
-      <c r="I7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="7" t="s">
+      <c r="D8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="9"/>
-      <c r="I8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="7" t="s">
+      <c r="D9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="9"/>
-      <c r="I9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="7" t="s">
+      <c r="D10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="9"/>
-      <c r="I10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="7" t="s">
+      <c r="D11" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="8" t="s">
         <v>13</v>
       </c>
       <c r="F11" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="I11" s="10"/>
+      <c r="I11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="7" t="s">
+      <c r="D12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="9"/>
-      <c r="I12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="6" t="s">
         <v>32</v>
       </c>
       <c r="C13" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="7" t="s">
+      <c r="D13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="9"/>
-      <c r="I13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>34</v>
       </c>
       <c r="C14" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="7" t="s">
+      <c r="D14" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H14" s="9"/>
-      <c r="I14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="n">
+      <c r="A15" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="7" t="s">
+      <c r="D15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H15" s="9"/>
-      <c r="I15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="n">
+      <c r="A16" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="7" t="s">
+      <c r="D16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H16" s="9"/>
-      <c r="I16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>40</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="7" t="s">
+      <c r="D17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="9"/>
-      <c r="I17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="n">
+      <c r="A18" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="6" t="s">
         <v>42</v>
       </c>
       <c r="C18" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="7" t="s">
+      <c r="D18" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="8" t="s">
         <v>13</v>
       </c>
       <c r="F18" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G18" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="H18" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="I18" s="10"/>
+      <c r="I18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>45</v>
       </c>
       <c r="C19" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="7" t="s">
+      <c r="D19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H19" s="9"/>
-      <c r="I19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="7" t="s">
+      <c r="D20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H20" s="9"/>
-      <c r="I20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="6" t="s">
         <v>49</v>
       </c>
       <c r="C21" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D21" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="7" t="s">
+      <c r="D21" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="G21" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H21" s="9"/>
-      <c r="I21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="6" t="s">
         <v>51</v>
       </c>
       <c r="C22" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="7" t="s">
+      <c r="D22" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="G22" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H22" s="9"/>
-      <c r="I22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="6" t="s">
         <v>53</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="7" t="s">
+      <c r="D23" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="G23" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H23" s="9"/>
-      <c r="I23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="6" t="s">
         <v>55</v>
       </c>
       <c r="C24" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="D24" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="7" t="s">
+      <c r="D24" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G24" s="9" t="s">
+      <c r="G24" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H24" s="9"/>
-      <c r="I24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="n">
+      <c r="A25" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D25" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="7" t="s">
+      <c r="D25" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H25" s="9"/>
-      <c r="I25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="6" t="s">
         <v>59</v>
       </c>
       <c r="C26" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="D26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="7" t="s">
+      <c r="D26" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="G26" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H26" s="9"/>
-      <c r="I26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="n">
+      <c r="A27" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="6" t="s">
         <v>61</v>
       </c>
       <c r="C27" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="7" t="s">
+      <c r="D27" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H27" s="9"/>
-      <c r="I27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="n">
+      <c r="A28" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="6" t="s">
         <v>63</v>
       </c>
       <c r="C28" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="D28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="7" t="s">
+      <c r="D28" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G28" s="9" t="s">
+      <c r="G28" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H28" s="9"/>
-      <c r="I28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="11"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F5:F28">
@@ -1708,8 +1802,8 @@
   <dimension ref="A1:I14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="0" width="12.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="36.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="1" width="12.97"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1780,29 +1874,33 @@
       <c r="H4" s="14"/>
       <c r="I4" s="14"/>
     </row>
-    <row r="5" customFormat="false" ht="15.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="n">
         <v>5</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-    </row>
-    <row r="6" customFormat="false" ht="15.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C5" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+    </row>
+    <row r="6" customFormat="false" ht="57.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="n">
         <v>6</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="C6" s="14"/>
+        <v>71</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>72</v>
+      </c>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
@@ -1815,10 +1913,10 @@
         <v>7</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
@@ -1827,116 +1925,124 @@
       <c r="H7" s="14"/>
       <c r="I7" s="14"/>
     </row>
-    <row r="8" customFormat="false" ht="28.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="57.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="n">
         <v>8</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
+        <v>75</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="B9" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
+      <c r="B9" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="n">
         <v>10</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
+        <v>79</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="n">
         <v>11</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+      <c r="C11" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="21"/>
+    </row>
+    <row r="12" customFormat="false" ht="43.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="n">
         <v>12</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>82</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="B13" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="n">
         <v>14</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="19"/>
+        <v>86</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -1973,101 +2079,107 @@
   <dimension ref="A1:I14"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="0" width="12.97"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="23" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="24" width="36.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="24" width="12.97"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="23" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B1" s="15" t="s">
+      <c r="A1" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="14" t="n">
+      <c r="C1" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
     </row>
     <row r="2" customFormat="false" ht="15.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="n">
+      <c r="A2" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
+      <c r="C2" s="26" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
     </row>
     <row r="3" customFormat="false" ht="15.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="n">
+      <c r="A3" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
     </row>
     <row r="4" customFormat="false" ht="15.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="n">
+      <c r="A4" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-    </row>
-    <row r="5" customFormat="false" ht="15.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="n">
+      <c r="C4" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+    </row>
+    <row r="5" customFormat="false" ht="15.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-    </row>
-    <row r="6" customFormat="false" ht="15.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="n">
+      <c r="C5" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+    </row>
+    <row r="6" customFormat="false" ht="57.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="C6" s="14"/>
+      <c r="B6" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>72</v>
+      </c>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
@@ -2076,132 +2188,140 @@
       <c r="I6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="56.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="n">
+      <c r="A7" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="C7" s="14" t="s">
+      <c r="B7" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+    </row>
+    <row r="8" customFormat="false" ht="57.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+    </row>
+    <row r="9" customFormat="false" ht="15.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+    </row>
+    <row r="10" customFormat="false" ht="15.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+    </row>
+    <row r="11" customFormat="false" ht="15.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+    </row>
+    <row r="12" customFormat="false" ht="43.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-    </row>
-    <row r="8" customFormat="false" ht="28.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-    </row>
-    <row r="9" customFormat="false" ht="15.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-    </row>
-    <row r="10" customFormat="false" ht="15.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-    </row>
-    <row r="11" customFormat="false" ht="15.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="n">
-        <v>11</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-    </row>
-    <row r="12" customFormat="false" ht="15.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-    </row>
-    <row r="13" customFormat="false" ht="15.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="n">
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
+    </row>
+    <row r="13" customFormat="false" ht="15.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="n">
         <v>13</v>
       </c>
-      <c r="B13" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-    </row>
-    <row r="14" customFormat="false" ht="15.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="n">
+      <c r="B13" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+    </row>
+    <row r="14" customFormat="false" ht="15.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="n">
         <v>14</v>
       </c>
-      <c r="B14" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="19"/>
+      <c r="B14" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -2239,28 +2359,28 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="22" t="s">
-        <v>84</v>
+      <c r="A1" s="31" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="32" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="24" t="s">
-        <v>85</v>
+      <c r="A3" s="33" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="34" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26" t="s">
-        <v>86</v>
+      <c r="A5" s="35" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>